<commit_message>
Actualización de interfaz en WOS: 'Discrepancias' y 'Auditar WOS'
</commit_message>
<xml_diff>
--- a/public/Formato_de_Carga_de_Personal.xlsx
+++ b/public/Formato_de_Carga_de_Personal.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+  <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Hermes Balza\Documents\Software\Logic Group Management\public\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Hermes Balza\Documents\Software\Logic Group Management\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -14,17 +14,12 @@
   <sheets>
     <sheet name="Personal" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-  </extLst>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="42">
   <si>
     <t>nombre</t>
   </si>
@@ -51,6 +46,105 @@
   </si>
   <si>
     <t>locationHistory</t>
+  </si>
+  <si>
+    <t>payer_type</t>
+  </si>
+  <si>
+    <t>tin_type</t>
+  </si>
+  <si>
+    <t>tin</t>
+  </si>
+  <si>
+    <t>first_name</t>
+  </si>
+  <si>
+    <t>last_name</t>
+  </si>
+  <si>
+    <t>address_1</t>
+  </si>
+  <si>
+    <t>city</t>
+  </si>
+  <si>
+    <t>state</t>
+  </si>
+  <si>
+    <t>zip</t>
+  </si>
+  <si>
+    <t>country</t>
+  </si>
+  <si>
+    <t>email_tax</t>
+  </si>
+  <si>
+    <t>site_code</t>
+  </si>
+  <si>
+    <t>Ejemplo Garcia</t>
+  </si>
+  <si>
+    <t>1010</t>
+  </si>
+  <si>
+    <t>01/01/2026</t>
+  </si>
+  <si>
+    <t>--</t>
+  </si>
+  <si>
+    <t>Janitorial</t>
+  </si>
+  <si>
+    <t>Sysco Arizona</t>
+  </si>
+  <si>
+    <t>Zelle: ejemplo@mail.com</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>[]</t>
+  </si>
+  <si>
+    <t>Individual</t>
+  </si>
+  <si>
+    <t>SSN</t>
+  </si>
+  <si>
+    <t>000-00-0000</t>
+  </si>
+  <si>
+    <t>Ejemplo</t>
+  </si>
+  <si>
+    <t>Garcia</t>
+  </si>
+  <si>
+    <t>123 Street Ave</t>
+  </si>
+  <si>
+    <t>Phoenix</t>
+  </si>
+  <si>
+    <t>AZ</t>
+  </si>
+  <si>
+    <t>85001</t>
+  </si>
+  <si>
+    <t>EE. UU.</t>
+  </si>
+  <si>
+    <t>ejemplo@mail.com</t>
+  </si>
+  <si>
+    <t>AZ-001</t>
   </si>
 </sst>
 </file>
@@ -59,7 +153,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
+      <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -67,10 +161,11 @@
     </font>
     <font>
       <b/>
-      <sz val="10"/>
+      <sz val="12"/>
       <color theme="1"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -81,7 +176,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -89,40 +184,19 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="medium">
-        <color rgb="FFCCCCCC"/>
-      </left>
-      <right style="medium">
-        <color rgb="FFCCCCCC"/>
-      </right>
-      <top style="medium">
-        <color rgb="FFCCCCCC"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FFCCCCCC"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+  <cellXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -135,7 +209,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -145,44 +219,44 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="44546A"/>
+        <a:srgbClr val="1F497D"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="E7E6E6"/>
+        <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="5B9BD5"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="ED7D31"/>
+        <a:srgbClr val="C0504D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="A5A5A5"/>
+        <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="FFC000"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4472C4"/>
+        <a:srgbClr val="4BACC6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="70AD47"/>
+        <a:srgbClr val="F79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0563C1"/>
+        <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="954F72"/>
+        <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック Light"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线 Light"/>
+        <a:font script="Hans" typeface="宋体"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
@@ -212,12 +286,12 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线"/>
+        <a:font script="Hans" typeface="宋体"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
@@ -256,160 +330,214 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:lumMod val="110000"/>
-                <a:satMod val="105000"/>
-                <a:tint val="67000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="103000"/>
-                <a:tint val="73000"/>
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="109000"/>
-                <a:tint val="81000"/>
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:satMod val="103000"/>
-                <a:lumMod val="102000"/>
-                <a:tint val="94000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:satMod val="110000"/>
-                <a:lumMod val="100000"/>
+                <a:tint val="100000"/>
                 <a:shade val="100000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="99000"/>
-                <a:satMod val="120000"/>
-                <a:shade val="78000"/>
+                <a:tint val="50000"/>
+                <a:shade val="100000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="16200000" scaled="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
         <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst/>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
-                <a:alpha val="63000"/>
+                <a:alpha val="35000"/>
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:tint val="95000"/>
-            <a:satMod val="170000"/>
-          </a:schemeClr>
-        </a:solidFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="93000"/>
-                <a:satMod val="150000"/>
-                <a:shade val="98000"/>
-                <a:lumMod val="102000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:tint val="98000"/>
-                <a:satMod val="130000"/>
-                <a:shade val="90000"/>
-                <a:lumMod val="103000"/>
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="40000">
+              <a:schemeClr val="phClr">
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="63000"/>
-                <a:satMod val="120000"/>
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
+  <a:objectDefaults>
+    <a:spDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="3">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </a:style>
+    </a:spDef>
+    <a:lnDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
   <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
-    </a:ext>
-  </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:U3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="37.42578125" customWidth="1"/>
-    <col min="2" max="2" width="18.7109375" style="3" customWidth="1"/>
-    <col min="3" max="9" width="18.7109375" customWidth="1"/>
-  </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:21" s="1" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
@@ -433,9 +561,114 @@
       <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>20</v>
+      </c>
     </row>
+    <row r="2" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D2" t="s">
+        <v>24</v>
+      </c>
+      <c r="E2" t="s">
+        <v>25</v>
+      </c>
+      <c r="F2" t="s">
+        <v>26</v>
+      </c>
+      <c r="G2" t="s">
+        <v>27</v>
+      </c>
+      <c r="H2" t="s">
+        <v>28</v>
+      </c>
+      <c r="I2" t="s">
+        <v>29</v>
+      </c>
+      <c r="J2" t="s">
+        <v>30</v>
+      </c>
+      <c r="K2" t="s">
+        <v>31</v>
+      </c>
+      <c r="L2" t="s">
+        <v>32</v>
+      </c>
+      <c r="M2" t="s">
+        <v>33</v>
+      </c>
+      <c r="N2" t="s">
+        <v>34</v>
+      </c>
+      <c r="O2" t="s">
+        <v>35</v>
+      </c>
+      <c r="P2" t="s">
+        <v>36</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>37</v>
+      </c>
+      <c r="R2" t="s">
+        <v>38</v>
+      </c>
+      <c r="S2" t="s">
+        <v>39</v>
+      </c>
+      <c r="T2" t="s">
+        <v>40</v>
+      </c>
+      <c r="U2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="3" spans="1:21" ht="15.75" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <ignoredErrors>
+    <ignoredError sqref="A1:U2" numberStoredAsText="1"/>
+  </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Agregar columnas Rate KBS, Rate LGM, Observaciones, Rate CSG y Cliente en plantilla de carga masiva de Personal
</commit_message>
<xml_diff>
--- a/public/Formato_de_Carga_de_Personal.xlsx
+++ b/public/Formato_de_Carga_de_Personal.xlsx
@@ -5,11 +5,11 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Hermes Balza\Documents\Software\Logic Group Management\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Hermes Balza\Documents\Software\Logic Group Management\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="8235"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="7770" windowHeight="4905"/>
   </bookViews>
   <sheets>
     <sheet name="Personal" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="50">
   <si>
     <t>nombre</t>
   </si>
@@ -84,6 +84,21 @@
     <t>site_code</t>
   </si>
   <si>
+    <t>Rate KBS</t>
+  </si>
+  <si>
+    <t>Rate LGM</t>
+  </si>
+  <si>
+    <t>Observaciones</t>
+  </si>
+  <si>
+    <t>Rate CSG</t>
+  </si>
+  <si>
+    <t>Cliente</t>
+  </si>
+  <si>
     <t>Ejemplo Garcia</t>
   </si>
   <si>
@@ -145,6 +160,15 @@
   </si>
   <si>
     <t>AZ-001</t>
+  </si>
+  <si>
+    <t>18.00</t>
+  </si>
+  <si>
+    <t>20.00</t>
+  </si>
+  <si>
+    <t>KBS</t>
   </si>
 </sst>
 </file>
@@ -530,10 +554,29 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:U3"/>
+  <dimension ref="A1:Z2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="12.875" customWidth="1"/>
+    <col min="2" max="2" width="19.875" customWidth="1"/>
+    <col min="3" max="3" width="17.875" customWidth="1"/>
+    <col min="4" max="4" width="16.875" customWidth="1"/>
+    <col min="5" max="6" width="12.875" customWidth="1"/>
+    <col min="7" max="7" width="19.875" customWidth="1"/>
+    <col min="8" max="8" width="12.875" customWidth="1"/>
+    <col min="9" max="9" width="19.875" customWidth="1"/>
+    <col min="10" max="10" width="14.875" customWidth="1"/>
+    <col min="11" max="12" width="12.875" customWidth="1"/>
+    <col min="13" max="13" width="14.875" customWidth="1"/>
+    <col min="14" max="15" width="13.875" customWidth="1"/>
+    <col min="16" max="19" width="12.875" customWidth="1"/>
+    <col min="20" max="21" width="13.875" customWidth="1"/>
+    <col min="22" max="23" width="12.875" customWidth="1"/>
+    <col min="24" max="24" width="17.875" customWidth="1"/>
+    <col min="25" max="26" width="12.875" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:21" s="1" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:26" s="1" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -597,78 +640,107 @@
       <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
+      <c r="V1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="X1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="Y1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Z1" s="1" t="s">
+        <v>25</v>
+      </c>
     </row>
-    <row r="2" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:26" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="B2" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="C2" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="D2" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="E2" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="F2" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="G2" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="H2" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="I2" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="J2" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="K2" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="L2" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="M2" t="s">
+        <v>38</v>
+      </c>
+      <c r="N2" t="s">
+        <v>39</v>
+      </c>
+      <c r="O2" t="s">
+        <v>40</v>
+      </c>
+      <c r="P2" t="s">
+        <v>41</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>42</v>
+      </c>
+      <c r="R2" t="s">
+        <v>43</v>
+      </c>
+      <c r="S2" t="s">
+        <v>44</v>
+      </c>
+      <c r="T2" t="s">
+        <v>45</v>
+      </c>
+      <c r="U2" t="s">
+        <v>46</v>
+      </c>
+      <c r="V2" t="s">
+        <v>47</v>
+      </c>
+      <c r="W2" t="s">
+        <v>48</v>
+      </c>
+      <c r="X2" t="s">
         <v>33</v>
       </c>
-      <c r="N2" t="s">
-        <v>34</v>
-      </c>
-      <c r="O2" t="s">
-        <v>35</v>
-      </c>
-      <c r="P2" t="s">
-        <v>36</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>37</v>
-      </c>
-      <c r="R2" t="s">
-        <v>38</v>
-      </c>
-      <c r="S2" t="s">
-        <v>39</v>
-      </c>
-      <c r="T2" t="s">
-        <v>40</v>
-      </c>
-      <c r="U2" t="s">
-        <v>41</v>
+      <c r="Y2" t="s">
+        <v>33</v>
+      </c>
+      <c r="Z2" t="s">
+        <v>49</v>
       </c>
     </row>
-    <row r="3" spans="1:21" ht="15.75" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:U2" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:Z2" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>